<commit_message>
Updating LCOH & emissions charts for MN fact sheet
</commit_message>
<xml_diff>
--- a/state_fact_sheets/data/modified/lcoh_policy_results.xlsx
+++ b/state_fact_sheets/data/modified/lcoh_policy_results.xlsx
@@ -375,7 +375,8 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share</t>
+          <t>Scenario 4 - 100% Capex
+Share</t>
         </is>
       </c>
     </row>
@@ -387,7 +388,8 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share</t>
+          <t>Scenario 4 - 100% Capex
+Share</t>
         </is>
       </c>
     </row>
@@ -399,7 +401,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate, Scenario 4 - No Policy</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate, Scenario 4 - No Policy</t>
         </is>
       </c>
     </row>
@@ -411,7 +417,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate, Scenario 4 - No Policy</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate, Scenario 4 - No Policy</t>
         </is>
       </c>
     </row>
@@ -423,7 +433,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate, Scenario 4 - No Policy</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate, Scenario 4 - No Policy</t>
         </is>
       </c>
     </row>
@@ -435,7 +449,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate, Scenario 4 - No Policy</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate, Scenario 4 - No Policy</t>
         </is>
       </c>
     </row>
@@ -447,7 +465,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate, Scenario 4 - No Policy</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate, Scenario 4 - No Policy</t>
         </is>
       </c>
     </row>
@@ -459,7 +481,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate, Scenario 4 - No Policy</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate, Scenario 4 - No Policy</t>
         </is>
       </c>
     </row>
@@ -471,7 +497,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate, Scenario 4 - No Policy</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate, Scenario 4 - No Policy</t>
         </is>
       </c>
     </row>
@@ -483,7 +513,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate, Scenario 4 - No Policy</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate, Scenario 4 - No Policy</t>
         </is>
       </c>
     </row>
@@ -495,7 +529,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate, Scenario 4 - No Policy</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate, Scenario 4 - No Policy</t>
         </is>
       </c>
     </row>
@@ -507,7 +545,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate, Scenario 4 - No Policy</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate, Scenario 4 - No Policy</t>
         </is>
       </c>
     </row>
@@ -519,7 +561,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate, Scenario 4 - No Policy</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate, Scenario 4 - No Policy</t>
         </is>
       </c>
     </row>
@@ -531,7 +577,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate, Scenario 4 - No Policy</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate, Scenario 4 - No Policy</t>
         </is>
       </c>
     </row>
@@ -543,7 +593,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate, Scenario 4 - No Policy</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate, Scenario 4 - No Policy</t>
         </is>
       </c>
     </row>
@@ -555,7 +609,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate, Scenario 4 - No Policy</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate, Scenario 4 - No Policy</t>
         </is>
       </c>
     </row>
@@ -567,7 +625,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate, Scenario 4 - No Policy</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate, Scenario 4 - No Policy</t>
         </is>
       </c>
     </row>
@@ -579,7 +641,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate, Scenario 4 - No Policy</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate, Scenario 4 - No Policy</t>
         </is>
       </c>
     </row>
@@ -591,7 +657,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate</t>
         </is>
       </c>
     </row>
@@ -603,7 +673,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 30% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate, Scenario 4 - No Policy</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 30% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate, Scenario 4 - No Policy</t>
         </is>
       </c>
     </row>
@@ -615,7 +689,8 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share</t>
+          <t>Scenario 4 - 100% Capex
+Share</t>
         </is>
       </c>
     </row>
@@ -639,7 +714,8 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share</t>
+          <t>Scenario 4 - 100% Capex
+Share</t>
         </is>
       </c>
     </row>
@@ -651,7 +727,10 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share, Scenario 4 - 50% Cost Share, Scenario 4 - Low Rate</t>
+          <t>Scenario 4 - 100% Capex
+Share, Scenario 4 - 50% Capex
+Share, Scenario 4 - Low Elec.
+Rate</t>
         </is>
       </c>
     </row>
@@ -673,22 +752,26 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Scenario 4 - 100% Cost Share</t>
+          <t>Scenario 4 - 100% Capex
+Share</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Scenario 4 - 50% Cost Share</t>
+          <t>Scenario 4 - 50% Capex
+Share</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Scenario 4 - Low Rate</t>
+          <t>Scenario 4 - Low Elec.
+Rate</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Scenario 4 - 30% Cost Share</t>
+          <t>Scenario 4 - 30% Capex
+Share</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>